<commit_message>
add Hogwarts to admin2 level to make clear demo data
</commit_message>
<xml_diff>
--- a/example_files/hmpv_metadata.xlsx
+++ b/example_files/hmpv_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aparker/Documents/Github/dev_example_data/example_files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emma\git_stuff\example_data\example_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B155EB39-1415-2440-A3D3-5BAAC3514E24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A476C0C-27CC-4B4D-8645-50577220ED1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{5AFB2170-2060-D54F-A32F-411131C97D7F}"/>
+    <workbookView xWindow="6120" yWindow="-19215" windowWidth="28800" windowHeight="15150" xr2:uid="{5AFB2170-2060-D54F-A32F-411131C97D7F}"/>
   </bookViews>
   <sheets>
     <sheet name="rsv_a_metadata" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
   <si>
     <t>submissionId</t>
   </si>
@@ -134,6 +134,9 @@
   </si>
   <si>
     <t>USA/WA-UW-1b519/2023</t>
+  </si>
+  <si>
+    <t>Hogwarts</t>
   </si>
 </sst>
 </file>
@@ -1010,12 +1013,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9376D926-3800-2A48-BB2C-D4DD0F811C1A}">
   <dimension ref="A1:X3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="23" max="23" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1089,7 +1092,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" ht="18" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -1102,6 +1105,9 @@
       <c r="E2" t="s">
         <v>34</v>
       </c>
+      <c r="F2" t="s">
+        <v>38</v>
+      </c>
       <c r="H2" s="1" t="s">
         <v>25</v>
       </c>
@@ -1121,7 +1127,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -1130,6 +1136,9 @@
       </c>
       <c r="C3" t="s">
         <v>28</v>
+      </c>
+      <c r="F3" t="s">
+        <v>38</v>
       </c>
       <c r="H3" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Update example data to use 'host' instead of 'hostTaxonId', 'hostNameScientific'
</commit_message>
<xml_diff>
--- a/example_files/hmpv_metadata.xlsx
+++ b/example_files/hmpv_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emma\git_stuff\example_data\example_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mverbies/projects/example_data/example_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A476C0C-27CC-4B4D-8645-50577220ED1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF78294-E71E-E845-9CC9-775DC6C8AB7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6120" yWindow="-19215" windowWidth="28800" windowHeight="15150" xr2:uid="{5AFB2170-2060-D54F-A32F-411131C97D7F}"/>
+    <workbookView xWindow="6120" yWindow="-19220" windowWidth="28800" windowHeight="15160" xr2:uid="{5AFB2170-2060-D54F-A32F-411131C97D7F}"/>
   </bookViews>
   <sheets>
     <sheet name="rsv_a_metadata" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="38">
   <si>
     <t>submissionId</t>
   </si>
@@ -58,12 +58,6 @@
     <t>hostAge</t>
   </si>
   <si>
-    <t>hostNameScientific</t>
-  </si>
-  <si>
-    <t>hostTaxonId</t>
-  </si>
-  <si>
     <t>insdcAccessionBase</t>
   </si>
   <si>
@@ -137,6 +131,9 @@
   </si>
   <si>
     <t>Hogwarts</t>
+  </si>
+  <si>
+    <t>host</t>
   </si>
 </sst>
 </file>
@@ -1012,13 +1009,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9376D926-3800-2A48-BB2C-D4DD0F811C1A}">
-  <dimension ref="A1:X3"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:W3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="23" max="23" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1056,107 +1053,104 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
+        <v>37</v>
+      </c>
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+    </row>
+    <row r="2" spans="1:23" ht="19" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
-        <v>23</v>
+      <c r="N2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V2" s="3">
+        <v>45092</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="18" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="3" spans="1:23" ht="18" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" t="s">
         <v>36</v>
       </c>
-      <c r="C2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H2" s="1" t="s">
+      <c r="H3" t="s">
+        <v>29</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" t="s">
         <v>25</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="O3" t="s">
         <v>24</v>
       </c>
-      <c r="O2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="P2" t="s">
-        <v>32</v>
-      </c>
-      <c r="W2" s="3">
-        <v>45092</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" ht="16.75" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="V3" s="3">
+        <v>45576</v>
+      </c>
+      <c r="W3" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="F3" t="s">
-        <v>38</v>
-      </c>
-      <c r="H3" t="s">
-        <v>31</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O3" t="s">
-        <v>27</v>
-      </c>
-      <c r="P3" t="s">
-        <v>26</v>
-      </c>
-      <c r="W3" s="3">
-        <v>45576</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>